<commit_message>
feat: implement SMRITI Retail OS v3.17.0 core UI/UX refactor, header mapping engine, and navigation shell updates
</commit_message>
<xml_diff>
--- a/SMRITI_Control_Plane_Architecture_Review.xlsx
+++ b/SMRITI_Control_Plane_Architecture_Review.xlsx
@@ -38781,7 +38781,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>45 Tables</t>
+          <t>99 Tables</t>
         </is>
       </c>
     </row>
@@ -38805,7 +38805,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>SalesInvoices=123, StockMovements=4</t>
+          <t>SalesInvoices=123, StockMovements=7</t>
         </is>
       </c>
     </row>

</xml_diff>